<commit_message>
canal-physical: make the comparison workbook reproducible
Two identical runs gave different bytes for comparison_all_images.xlsx, and only
that file. openpyxl writes the time of saving into docProps/core.xml whatever the
document properties say, and gives every zip entry the current time.

The workbook is now rewritten after saving with fixed entry dates and a fixed
created and modified stamp, so the file depends on the numbers in it and nothing
else. The cell values are copied untouched. The csv and the pdf were already
reproducible, and the png and pdf figures had their timestamps suppressed
earlier.

Verified in isolation: the workbook written twice, a second apart, is byte
identical, as are the csv and the pdf.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results_experiments/canal_physical/comparison_all_images.xlsx
+++ b/results_experiments/canal_physical/comparison_all_images.xlsx
@@ -2628,7 +2628,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>128.476517</v>
+        <v>14.912426</v>
       </c>
       <c r="E3" t="n">
         <v>25</v>
@@ -2643,12 +2643,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>above</t>
+          <t>below</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>a 3D length; a 2D section holds only part of a thread</t>
+          <t>owned length per cell divided by roots per cell; a 2D section holds only part of a thread, and ownership has no distance limit</t>
         </is>
       </c>
     </row>
@@ -2792,7 +2792,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>276.782103</v>
+        <v>25.162009</v>
       </c>
       <c r="E7" t="n">
         <v>25</v>
@@ -2807,12 +2807,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>above</t>
+          <t>inside</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>a 3D length; a 2D section holds only part of a thread</t>
+          <t>owned length per cell divided by roots per cell; a 2D section holds only part of a thread, and ownership has no distance limit</t>
         </is>
       </c>
     </row>
@@ -2956,7 +2956,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>126.439989</v>
+        <v>15.284005</v>
       </c>
       <c r="E11" t="n">
         <v>25</v>
@@ -2971,12 +2971,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>above</t>
+          <t>below</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>a 3D length; a 2D section holds only part of a thread</t>
+          <t>owned length per cell divided by roots per cell; a 2D section holds only part of a thread, and ownership has no distance limit</t>
         </is>
       </c>
     </row>
@@ -3120,7 +3120,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>310.179688</v>
+        <v>36.29743</v>
       </c>
       <c r="E15" t="n">
         <v>25</v>
@@ -3135,12 +3135,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>above</t>
+          <t>inside</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>a 3D length; a 2D section holds only part of a thread</t>
+          <t>owned length per cell divided by roots per cell; a 2D section holds only part of a thread, and ownership has no distance limit</t>
         </is>
       </c>
     </row>
@@ -3284,7 +3284,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>219.353264</v>
+        <v>28.925832</v>
       </c>
       <c r="E19" t="n">
         <v>25</v>
@@ -3299,12 +3299,12 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>above</t>
+          <t>inside</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>a 3D length; a 2D section holds only part of a thread</t>
+          <t>owned length per cell divided by roots per cell; a 2D section holds only part of a thread, and ownership has no distance limit</t>
         </is>
       </c>
     </row>
@@ -3448,7 +3448,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>454.531038</v>
+        <v>65.715014</v>
       </c>
       <c r="E23" t="n">
         <v>25</v>
@@ -3468,7 +3468,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>a 3D length; a 2D section holds only part of a thread</t>
+          <t>owned length per cell divided by roots per cell; a 2D section holds only part of a thread, and ownership has no distance limit</t>
         </is>
       </c>
     </row>
@@ -3612,7 +3612,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>186.569097</v>
+        <v>27.082567</v>
       </c>
       <c r="E27" t="n">
         <v>25</v>
@@ -3627,12 +3627,12 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>above</t>
+          <t>inside</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>a 3D length; a 2D section holds only part of a thread</t>
+          <t>owned length per cell divided by roots per cell; a 2D section holds only part of a thread, and ownership has no distance limit</t>
         </is>
       </c>
     </row>
@@ -3776,7 +3776,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>590.5319940000001</v>
+        <v>83.043691</v>
       </c>
       <c r="E31" t="n">
         <v>25</v>
@@ -3796,7 +3796,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>a 3D length; a 2D section holds only part of a thread</t>
+          <t>owned length per cell divided by roots per cell; a 2D section holds only part of a thread, and ownership has no distance limit</t>
         </is>
       </c>
     </row>
@@ -3940,7 +3940,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>222.818258</v>
+        <v>33.121499</v>
       </c>
       <c r="E35" t="n">
         <v>25</v>
@@ -3955,12 +3955,12 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>above</t>
+          <t>inside</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>a 3D length; a 2D section holds only part of a thread</t>
+          <t>owned length per cell divided by roots per cell; a 2D section holds only part of a thread, and ownership has no distance limit</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>397.98655</v>
+        <v>62.541101</v>
       </c>
       <c r="E39" t="n">
         <v>25</v>
@@ -4124,7 +4124,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>a 3D length; a 2D section holds only part of a thread</t>
+          <t>owned length per cell divided by roots per cell; a 2D section holds only part of a thread, and ownership has no distance limit</t>
         </is>
       </c>
     </row>
@@ -4268,7 +4268,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>241.872943</v>
+        <v>24.187294</v>
       </c>
       <c r="E43" t="n">
         <v>25</v>
@@ -4283,12 +4283,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>above</t>
+          <t>below</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>a 3D length; a 2D section holds only part of a thread</t>
+          <t>owned length per cell divided by roots per cell; a 2D section holds only part of a thread, and ownership has no distance limit</t>
         </is>
       </c>
     </row>
@@ -4432,7 +4432,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>443.696565</v>
+        <v>41.759677</v>
       </c>
       <c r="E47" t="n">
         <v>25</v>
@@ -4447,12 +4447,12 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>above</t>
+          <t>inside</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>a 3D length; a 2D section holds only part of a thread</t>
+          <t>owned length per cell divided by roots per cell; a 2D section holds only part of a thread, and ownership has no distance limit</t>
         </is>
       </c>
     </row>
@@ -4596,7 +4596,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>138.556184</v>
+        <v>20.596106</v>
       </c>
       <c r="E51" t="n">
         <v>25</v>
@@ -4611,12 +4611,12 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>above</t>
+          <t>below</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>a 3D length; a 2D section holds only part of a thread</t>
+          <t>owned length per cell divided by roots per cell; a 2D section holds only part of a thread, and ownership has no distance limit</t>
         </is>
       </c>
     </row>
@@ -4760,7 +4760,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>310.433409</v>
+        <v>45.530112</v>
       </c>
       <c r="E55" t="n">
         <v>25</v>
@@ -4775,12 +4775,12 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>above</t>
+          <t>inside</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>a 3D length; a 2D section holds only part of a thread</t>
+          <t>owned length per cell divided by roots per cell; a 2D section holds only part of a thread, and ownership has no distance limit</t>
         </is>
       </c>
     </row>
@@ -4924,7 +4924,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>110.306898</v>
+        <v>19.891245</v>
       </c>
       <c r="E59" t="n">
         <v>25</v>
@@ -4939,12 +4939,12 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>above</t>
+          <t>below</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>a 3D length; a 2D section holds only part of a thread</t>
+          <t>owned length per cell divided by roots per cell; a 2D section holds only part of a thread, and ownership has no distance limit</t>
         </is>
       </c>
     </row>
@@ -5088,7 +5088,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>337.023791</v>
+        <v>62.83537</v>
       </c>
       <c r="E63" t="n">
         <v>25</v>
@@ -5108,7 +5108,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>a 3D length; a 2D section holds only part of a thread</t>
+          <t>owned length per cell divided by roots per cell; a 2D section holds only part of a thread, and ownership has no distance limit</t>
         </is>
       </c>
     </row>

</xml_diff>